<commit_message>
Daily job match 2026-08-03
</commit_message>
<xml_diff>
--- a/output/matches_2026-08-03.xlsx
+++ b/output/matches_2026-08-03.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,7 +474,127 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.com/land/ad/5748993355?se=rLxEIVmP8RGMVoxu7ge2EQ&amp;utm_medium=api&amp;utm_source=c998f847&amp;v=5B16C3053C01862EF92DC23FA2C9085FF09628CB</t>
+          <t>https://www.adzuna.com/land/ad/5748993355?se=TqhjZF-P8RGSKpdiNYykDw&amp;utm_medium=api&amp;utm_source=c998f847&amp;v=5B16C3053C01862EF92DC23FA2C9085FF09628CB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Head of Post-Sales Technical Solutions (Miami)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Ramp</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Brickell, Miami-Dade County</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>technical consulting, onboarding, SaaS</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.com/land/ad/5814013100?se=ttX-ZV-P8RG0dPTDkKw-Ag&amp;utm_medium=api&amp;utm_source=c998f847&amp;v=8CEDE4C2ABEB46D5CFDBADA54858324368E18045</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Braze Migration Support</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Digital</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Miami, Miami-Dade County</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>technical consulting, Salesforce</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.com/details/5826553779?utm_medium=api&amp;utm_source=c998f847</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SQL DBA / Systems Analyst</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Contact Government Services</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Miami, Miami-Dade County</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SQL, technical support</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.com/land/ad/5675791814?se=ttX-ZV-P8RG0dPTDkKw-Ag&amp;utm_medium=api&amp;utm_source=c998f847&amp;v=610E7E521ED8D4538CFE5FB51E84C0B508A35CF8</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Project Manager (Bay Pines, FL)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Planate Management Group</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Brickell, Miami-Dade County</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>technical support, technical consulting</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.adzuna.com/details/5658621191?utm_medium=api&amp;utm_source=c998f847</t>
         </is>
       </c>
     </row>

</xml_diff>